<commit_message>
On branch master Your branch is up to date with 'origin/master'.
Changes to be committed:
	modified:   other/MarayaEngreering/Touch_zone/Touch_zone.xlsx
	new file:   other/MarayaEngreering/access-card_permissions_enable-disable.txt
</commit_message>
<xml_diff>
--- a/other/MarayaEngreering/Touch_zone/Touch_zone.xlsx
+++ b/other/MarayaEngreering/Touch_zone/Touch_zone.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\myGit\cheatsheets\other\MarayaEngreering\Touch_zone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CA0CF40-36FA-40DC-A8C6-AE902718D0EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88D05B91-AAD0-4B38-92BA-9EE6882771D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="47">
   <si>
     <t>TOUCH ZONE 5 (IP 10.4.101.8)</t>
   </si>
@@ -39,9 +39,6 @@
     <t>VIP GREENROOM ON/OFF</t>
   </si>
   <si>
-    <t>GROUND FOOR</t>
-  </si>
-  <si>
     <t>VIP GREENROOM COVE ON/OFF</t>
   </si>
   <si>
@@ -112,6 +109,66 @@
   </si>
   <si>
     <t>FIRST FOOR</t>
+  </si>
+  <si>
+    <t>GROUND FOOR = GndF</t>
+  </si>
+  <si>
+    <t>THIRD FOOR = 3rdF</t>
+  </si>
+  <si>
+    <t>BAR &amp; RESTAURANT</t>
+  </si>
+  <si>
+    <t>BAR &amp; RESTAURANT ON/OFF</t>
+  </si>
+  <si>
+    <t>TOILETS ON/OFF</t>
+  </si>
+  <si>
+    <t>Off</t>
+  </si>
+  <si>
+    <t>GF RESTAURANT</t>
+  </si>
+  <si>
+    <t>RESTAURANT AREA ON/OFF</t>
+  </si>
+  <si>
+    <t>RESTAURANT LOW CEILLING SPOT ON/OFF</t>
+  </si>
+  <si>
+    <t>RESTAURANT LOW CEILLING DIM</t>
+  </si>
+  <si>
+    <t>RESTAURANT HIGH CEILING TRACK ON/OFF</t>
+  </si>
+  <si>
+    <t>RESTAURANT HIGH CEILING DECORATIVE SUSPENSON ON/OFF</t>
+  </si>
+  <si>
+    <t>RESTAURANT AREA FOLIO 4000K ON/OFF</t>
+  </si>
+  <si>
+    <t>RESTAURANT AREA FOLIO 3200K ON/OFF</t>
+  </si>
+  <si>
+    <t>RESTAURANT AREA COVE LIGHTS ON/OFF</t>
+  </si>
+  <si>
+    <t>RESTAURANT LOW CEILING TRACK ON/OFF</t>
+  </si>
+  <si>
+    <t>RESTAURANT LOW CEILING DECORATIVE SUSPENSION ON/OFF</t>
+  </si>
+  <si>
+    <t>RESTAURANT HIGH CEILING AREA DIM</t>
+  </si>
+  <si>
+    <t>RESTAURANT AREA FOLIO 2700K ON/OFF</t>
+  </si>
+  <si>
+    <t>RESTAURANT AREA FOLIO 4000K DIM</t>
   </si>
 </sst>
 </file>
@@ -197,17 +254,17 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -489,30 +546,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B87"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="44.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="53.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="25.8" x14ac:dyDescent="0.5">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
+      <c r="B1" s="5"/>
     </row>
     <row r="2" spans="1:2" ht="21" x14ac:dyDescent="0.4">
-      <c r="A2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="4"/>
+      <c r="A2" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="6"/>
     </row>
     <row r="3" spans="1:2" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>13</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -520,7 +577,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -528,28 +585,28 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8" s="2">
         <v>0.75</v>
@@ -557,47 +614,47 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B14" s="2">
         <v>0.25</v>
@@ -605,102 +662,268 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A25" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" s="6"/>
+    </row>
+    <row r="26" spans="1:2" ht="18" x14ac:dyDescent="0.35">
+      <c r="A26" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>37</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>41</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>42</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>43</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>44</v>
+      </c>
+      <c r="B37" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>45</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>46</v>
+      </c>
+      <c r="B39" s="2">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A75" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="21" x14ac:dyDescent="0.4">
-      <c r="A25" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B25" s="4"/>
-    </row>
-    <row r="26" spans="1:2" ht="18" x14ac:dyDescent="0.35">
-      <c r="A26" s="5" t="s">
+      <c r="B75" s="6"/>
+    </row>
+    <row r="76" spans="1:2" ht="18" x14ac:dyDescent="0.35">
+      <c r="A76" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B76" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="6" t="s">
-        <v>14</v>
+    </row>
+    <row r="82" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A82" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B82" s="6"/>
+    </row>
+    <row r="83" spans="1:2" ht="18" x14ac:dyDescent="0.35">
+      <c r="A83" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>30</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>5</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>29</v>
+      </c>
+      <c r="B86" s="2">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>31</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A75:B75"/>
+    <mergeCell ref="A82:B82"/>
     <mergeCell ref="A25:B25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>